<commit_message>
feat: importacao de pacientes via planilha aceita CPF e RG
Estende o mapeamento de colunas (CPF, RG - Numero, Data de Expedicao,
Orgao Emissor) e a planilha modelo publicada. dependente/responsavel
financeiro ficam de fora por decisao explicita (nao ha como referenciar
outro paciente por texto na planilha sem reintroduzir a ambiguidade de
matching por nome ja descartada pro Consultorio/Pacote).
</commit_message>
<xml_diff>
--- a/web/public/planilha-modelo-pacientes.xlsx
+++ b/web/public/planilha-modelo-pacientes.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:L2"/>
   <cols>
     <col min="1" max="1" width="24.83203125" customWidth="1"/>
     <col min="2" max="2" width="24.83203125" customWidth="1"/>
@@ -407,6 +407,10 @@
     <col min="6" max="6" width="24.83203125" customWidth="1"/>
     <col min="7" max="7" width="24.83203125" customWidth="1"/>
     <col min="8" max="8" width="24.83203125" customWidth="1"/>
+    <col min="9" max="9" width="24.83203125" customWidth="1"/>
+    <col min="10" max="10" width="24.83203125" customWidth="1"/>
+    <col min="11" max="11" width="24.83203125" customWidth="1"/>
+    <col min="12" max="12" width="24.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -434,6 +438,18 @@
       <c r="H1" t="str">
         <v>Precisa de recibo</v>
       </c>
+      <c r="I1" t="str">
+        <v>CPF</v>
+      </c>
+      <c r="J1" t="str">
+        <v>RG - Número</v>
+      </c>
+      <c r="K1" t="str">
+        <v>Data de Expedição (RG)</v>
+      </c>
+      <c r="L1" t="str">
+        <v>Órgão Emissor (RG)</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -460,10 +476,22 @@
       <c r="H2" t="str">
         <v>Sim</v>
       </c>
+      <c r="I2" t="str">
+        <v>111.222.333-44</v>
+      </c>
+      <c r="J2" t="str">
+        <v>MG-12.345.678</v>
+      </c>
+      <c r="K2" t="str">
+        <v>10/05/2015</v>
+      </c>
+      <c r="L2" t="str">
+        <v>SSP</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: import por planilha aceita campo Documento (Receita Saude/Nota Fiscal)
</commit_message>
<xml_diff>
--- a/web/public/planilha-modelo-pacientes.xlsx
+++ b/web/public/planilha-modelo-pacientes.xlsx
@@ -436,7 +436,7 @@
         <v>Observações</v>
       </c>
       <c r="H1" t="str">
-        <v>Precisa de recibo</v>
+        <v>Documento</v>
       </c>
       <c r="I1" t="str">
         <v>CPF</v>
@@ -474,7 +474,7 @@
         <v>Paciente encaminhada pelo Dr. João</v>
       </c>
       <c r="H2" t="str">
-        <v>Sim</v>
+        <v>Receita Saúde</v>
       </c>
       <c r="I2" t="str">
         <v>111.222.333-44</v>

</xml_diff>